<commit_message>
Correct Ali's date of birth
</commit_message>
<xml_diff>
--- a/Grubbins-data.xlsx
+++ b/Grubbins-data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/victoriagibbs/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/victoriagibbs/Documents/Project Grubbins/Family-dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BCB37EEB-20C8-3348-8E6A-040B4A9B7D87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20425D9D-8946-E14C-8623-F47072194CB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21780" yWindow="9640" windowWidth="32260" windowHeight="25460" activeTab="1" xr2:uid="{800D77CF-647F-E34B-8185-798B0D421593}"/>
+    <workbookView xWindow="4300" yWindow="780" windowWidth="29900" windowHeight="19660" activeTab="1" xr2:uid="{800D77CF-647F-E34B-8185-798B0D421593}"/>
   </bookViews>
   <sheets>
     <sheet name="Quotes" sheetId="1" r:id="rId1"/>
@@ -471,7 +471,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -481,7 +481,6 @@
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="16" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -966,7 +965,7 @@
         <v>32</v>
       </c>
       <c r="C2" s="4">
-        <v>30489</v>
+        <v>29759</v>
       </c>
       <c r="D2" t="s">
         <v>33</v>
@@ -1492,7 +1491,7 @@
       <c r="B40" t="s">
         <v>45</v>
       </c>
-      <c r="C40" s="9">
+      <c r="C40" s="4">
         <v>41845</v>
       </c>
       <c r="D40" t="s">
@@ -1506,7 +1505,7 @@
       <c r="B41" t="s">
         <v>46</v>
       </c>
-      <c r="C41" s="9">
+      <c r="C41" s="4">
         <v>41845</v>
       </c>
       <c r="D41" t="s">

</xml_diff>

<commit_message>
Update Important Dates and add Snoopy images
</commit_message>
<xml_diff>
--- a/Grubbins-data.xlsx
+++ b/Grubbins-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/victoriagibbs/Documents/Project Grubbins/Family-dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0939061F-1D58-F54D-A28A-C25A2FCAC118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A20B60F7-BB91-354D-AC25-2FAE694935AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4300" yWindow="780" windowWidth="29900" windowHeight="19660" activeTab="1" xr2:uid="{800D77CF-647F-E34B-8185-798B0D421593}"/>
   </bookViews>
@@ -286,18 +286,6 @@
     <t>nana-mary</t>
   </si>
   <si>
-    <t>markus</t>
-  </si>
-  <si>
-    <t>elizabeth</t>
-  </si>
-  <si>
-    <t>victoria</t>
-  </si>
-  <si>
-    <t>dave</t>
-  </si>
-  <si>
     <t>Markus</t>
   </si>
   <si>
@@ -422,6 +410,18 @@
   </si>
   <si>
     <t>Shaun</t>
+  </si>
+  <si>
+    <t>victoriaTruth</t>
+  </si>
+  <si>
+    <t>daveTruth</t>
+  </si>
+  <si>
+    <t>elizabethTruth</t>
+  </si>
+  <si>
+    <t>markusTruth</t>
   </si>
 </sst>
 </file>
@@ -483,14 +483,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1151,7 +1150,7 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B15" t="s">
         <v>46</v>
@@ -1291,10 +1290,10 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
+        <v>126</v>
+      </c>
+      <c r="B25" t="s">
         <v>81</v>
-      </c>
-      <c r="B25" t="s">
-        <v>85</v>
       </c>
       <c r="C25" s="3">
         <v>45763</v>
@@ -1305,10 +1304,10 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
+        <v>125</v>
+      </c>
+      <c r="B26" t="s">
         <v>82</v>
-      </c>
-      <c r="B26" t="s">
-        <v>86</v>
       </c>
       <c r="C26" s="3">
         <v>43363</v>
@@ -1319,10 +1318,10 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
+        <v>123</v>
+      </c>
+      <c r="B27" t="s">
         <v>83</v>
-      </c>
-      <c r="B27" t="s">
-        <v>87</v>
       </c>
       <c r="C27" s="3">
         <v>30431</v>
@@ -1333,10 +1332,10 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
+        <v>124</v>
+      </c>
+      <c r="B28" t="s">
         <v>84</v>
-      </c>
-      <c r="B28" t="s">
-        <v>88</v>
       </c>
       <c r="C28" s="3">
         <v>30416</v>
@@ -1347,66 +1346,66 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
+        <v>124</v>
+      </c>
+      <c r="B29" t="s">
         <v>84</v>
-      </c>
-      <c r="B29" t="s">
-        <v>88</v>
       </c>
       <c r="C29" s="3">
         <v>42595</v>
       </c>
       <c r="D29" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
+        <v>123</v>
+      </c>
+      <c r="B30" t="s">
         <v>83</v>
-      </c>
-      <c r="B30" t="s">
-        <v>87</v>
       </c>
       <c r="C30" s="3">
         <v>42595</v>
       </c>
       <c r="D30" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B31" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C31" s="3">
         <v>42119</v>
       </c>
       <c r="D31" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B32" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C32" s="3">
         <v>42119</v>
       </c>
       <c r="D32" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B33" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C33" s="3">
         <v>30482</v>
@@ -1420,13 +1419,13 @@
         <v>59</v>
       </c>
       <c r="B34" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C34" s="3">
         <v>39267</v>
       </c>
       <c r="D34" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -1434,21 +1433,21 @@
         <v>60</v>
       </c>
       <c r="B35" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C35" s="3">
         <v>39267</v>
       </c>
       <c r="D35" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B36" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C36" s="5">
         <v>160</v>
@@ -1468,7 +1467,7 @@
         <v>206</v>
       </c>
       <c r="D37" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -1482,15 +1481,15 @@
         <v>206</v>
       </c>
       <c r="D38" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B39" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C39" s="5">
         <v>207</v>
@@ -1510,12 +1509,12 @@
         <v>41845</v>
       </c>
       <c r="D40" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B41" t="s">
         <v>46</v>
@@ -1524,7 +1523,7 @@
         <v>41845</v>
       </c>
       <c r="D41" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -1538,7 +1537,7 @@
         <v>29428</v>
       </c>
       <c r="D42" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -1552,15 +1551,15 @@
         <v>29428</v>
       </c>
       <c r="D43" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B44" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C44" s="3">
         <v>41465</v>
@@ -1571,10 +1570,10 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B45" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C45" s="3">
         <v>30532</v>
@@ -1594,7 +1593,7 @@
         <v>39298</v>
       </c>
       <c r="D46" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -1608,15 +1607,15 @@
         <v>39298</v>
       </c>
       <c r="D47" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B48" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C48" s="3">
         <v>30578</v>
@@ -1627,10 +1626,10 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B49" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C49" s="3">
         <v>30623</v>
@@ -1641,10 +1640,10 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B50" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C50" s="3">
         <v>30670</v>
@@ -1655,10 +1654,10 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B51" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C51" s="5">
         <v>30</v>
@@ -1669,10 +1668,10 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B52" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C52" s="5">
         <v>95</v>
@@ -1683,10 +1682,10 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B53" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C53" s="3">
         <v>30422</v>
@@ -1697,10 +1696,10 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B54" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C54" s="3">
         <v>40658</v>
@@ -1711,10 +1710,10 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B55" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C55" s="5">
         <v>120</v>
@@ -1725,12 +1724,12 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B56" t="s">
-        <v>122</v>
-      </c>
-      <c r="C56" s="6">
+        <v>118</v>
+      </c>
+      <c r="C56" s="3">
         <v>30461</v>
       </c>
       <c r="D56" t="s">
@@ -1739,10 +1738,10 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B57" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C57" s="3">
         <v>30302</v>
@@ -1753,10 +1752,10 @@
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B58" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C58" s="5">
         <v>30529</v>

</xml_diff>